<commit_message>
excel observation entries for land use/cover
</commit_message>
<xml_diff>
--- a/lucas/import_data/utility/observation/excel/analysis_method.xlsx
+++ b/lucas/import_data/utility/observation/excel/analysis_method.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="191">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -584,6 +584,15 @@
   </si>
   <si>
     <t xml:space="preserve">Exchangable cations ammonium acetate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">derived</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Derived</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Derived nominative classification from one or more numerical values</t>
   </si>
 </sst>
 </file>
@@ -594,7 +603,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="[hh]:mm:ss"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -615,11 +624,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -704,7 +708,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -713,11 +717,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -737,15 +745,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -833,37 +833,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -936,8 +936,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F71"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="36.55"/>
@@ -1570,10 +1570,10 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8" t="s">
+      <c r="A33" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="2" t="s">
         <v>93</v>
       </c>
       <c r="C33" s="1" t="s">
@@ -1610,10 +1610,10 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="8" t="s">
+      <c r="A35" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="2" t="s">
         <v>95</v>
       </c>
       <c r="C35" s="1" t="s">
@@ -1650,10 +1650,10 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="8" t="s">
+      <c r="A37" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B37" s="8" t="s">
+      <c r="B37" s="2" t="s">
         <v>97</v>
       </c>
       <c r="C37" s="1" t="s">
@@ -1670,10 +1670,10 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="8" t="s">
+      <c r="A38" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="2" t="s">
         <v>100</v>
       </c>
       <c r="C38" s="1" t="s">
@@ -1685,15 +1685,15 @@
       <c r="E38" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F38" s="8" t="s">
+      <c r="F38" s="2" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="8" t="s">
+      <c r="A39" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B39" s="8" t="s">
+      <c r="B39" s="2" t="s">
         <v>101</v>
       </c>
       <c r="C39" s="1" t="s">
@@ -1705,7 +1705,7 @@
       <c r="E39" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F39" s="8" t="s">
+      <c r="F39" s="2" t="s">
         <v>99</v>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
       <c r="E53" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F53" s="8" t="s">
+      <c r="F53" s="2" t="s">
         <v>142</v>
       </c>
     </row>
@@ -2010,10 +2010,10 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="9" t="s">
+      <c r="A55" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="B55" s="9" t="s">
+      <c r="B55" s="8" t="s">
         <v>147</v>
       </c>
       <c r="C55" s="1" t="s">
@@ -2025,7 +2025,7 @@
       <c r="E55" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F55" s="9" t="s">
+      <c r="F55" s="8" t="s">
         <v>148</v>
       </c>
     </row>
@@ -2050,7 +2050,7 @@
       <c r="A57" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="B57" s="8" t="s">
+      <c r="B57" s="2" t="s">
         <v>152</v>
       </c>
       <c r="C57" s="1" t="s">
@@ -2062,7 +2062,7 @@
       <c r="E57" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F57" s="10" t="s">
+      <c r="F57" s="9" t="s">
         <v>153</v>
       </c>
     </row>
@@ -2070,7 +2070,7 @@
       <c r="A58" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="B58" s="8" t="s">
+      <c r="B58" s="2" t="s">
         <v>155</v>
       </c>
       <c r="C58" s="1" t="s">
@@ -2082,7 +2082,7 @@
       <c r="E58" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F58" s="10" t="s">
+      <c r="F58" s="9" t="s">
         <v>153</v>
       </c>
     </row>
@@ -2090,7 +2090,7 @@
       <c r="A59" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B59" s="8" t="s">
+      <c r="B59" s="2" t="s">
         <v>157</v>
       </c>
       <c r="C59" s="1" t="s">
@@ -2127,10 +2127,10 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="8" t="s">
+      <c r="A61" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B61" s="8" t="s">
+      <c r="B61" s="2" t="s">
         <v>163</v>
       </c>
       <c r="C61" s="1" t="s">
@@ -2147,10 +2147,10 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="9" t="s">
+      <c r="A62" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="B62" s="9" t="s">
+      <c r="B62" s="8" t="s">
         <v>165</v>
       </c>
       <c r="C62" s="1" t="s">
@@ -2162,7 +2162,7 @@
       <c r="E62" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F62" s="9" t="s">
+      <c r="F62" s="8" t="s">
         <v>166</v>
       </c>
     </row>
@@ -2187,7 +2187,7 @@
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="8" t="s">
+      <c r="A64" s="2" t="s">
         <v>170</v>
       </c>
       <c r="B64" s="1" t="s">
@@ -2210,7 +2210,7 @@
       <c r="A65" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="B65" s="8" t="s">
+      <c r="B65" s="2" t="s">
         <v>172</v>
       </c>
       <c r="C65" s="1" t="s">
@@ -2222,7 +2222,7 @@
       <c r="E65" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F65" s="8" t="s">
+      <c r="F65" s="2" t="s">
         <v>173</v>
       </c>
     </row>
@@ -2262,21 +2262,21 @@
       <c r="E67" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F67" s="8" t="s">
+      <c r="F67" s="2" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="8" t="s">
+      <c r="A68" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="B68" s="11" t="s">
+      <c r="B68" s="10" t="s">
         <v>179</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D68" s="11" t="s">
+      <c r="D68" s="10" t="s">
         <v>180</v>
       </c>
       <c r="E68" s="1" t="s">
@@ -2290,7 +2290,7 @@
       <c r="A69" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="B69" s="8" t="s">
+      <c r="B69" s="2" t="s">
         <v>183</v>
       </c>
       <c r="C69" s="1" t="s">
@@ -2307,7 +2307,7 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="8" t="s">
+      <c r="A70" s="2" t="s">
         <v>186</v>
       </c>
       <c r="B70" s="1" t="s">
@@ -2322,8 +2322,28 @@
       <c r="E70" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="F70" s="8" t="s">
+      <c r="F70" s="2" t="s">
         <v>185</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>